<commit_message>
Daily attendance processing - 2026-06-11 00:07:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -9012,7 +9012,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027</t>
+          <t>2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -12246,7 +12246,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-17 00:11:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -8960,7 +8960,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027</t>
+          <t>2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -12178,7 +12178,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-18 10:05:48 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -8948,7 +8948,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028</t>
+          <t>2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -12162,7 +12162,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-20 23:55:43 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -8936,7 +8936,7 @@
       </c>
       <c r="G180" s="4" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027</t>
+          <t>2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H180" s="4" t="inlineStr">
@@ -12142,7 +12142,7 @@
       </c>
       <c r="G250" s="4" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H250" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-22 18:24:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -8912,7 +8912,7 @@
       </c>
       <c r="G180" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027</t>
+          <t>2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H180" s="5" t="inlineStr">
@@ -12098,7 +12098,7 @@
       </c>
       <c r="G250" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H250" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-23 09:46:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -8904,7 +8904,7 @@
       </c>
       <c r="G180" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027</t>
+          <t>2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H180" s="5" t="inlineStr">
@@ -12078,7 +12078,7 @@
       </c>
       <c r="G250" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H250" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-28 01:47:33 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7">
@@ -842,53 +842,49 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>29/12/2025</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>66/66</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>0/66</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -953,7 +949,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>41.9%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1006,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>75.2%</t>
         </is>
       </c>
     </row>
@@ -1311,22 +1307,22 @@
         <v>53</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>39.6%</t>
+          <t>37.7%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>79.1%</t>
+          <t>78.0%</t>
         </is>
       </c>
     </row>
@@ -1475,22 +1471,22 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>41.5%</t>
+          <t>39.6%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>72.4%</t>
+          <t>71.4%</t>
         </is>
       </c>
     </row>
@@ -1557,22 +1553,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>48.1%</t>
+          <t>46.2%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>72.1%</t>
+          <t>74.4%</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1635,22 @@
         <v>54</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>70.2%</t>
+          <t>70.3%</t>
         </is>
       </c>
     </row>
@@ -7811,49 +7807,45 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B157" s="5" t="inlineStr">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C157" s="5" t="inlineStr">
+      <c r="C157" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D157" s="5" t="inlineStr">
+      <c r="D157" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E157" s="5" t="inlineStr">
+      <c r="E157" s="2" t="inlineStr">
         <is>
           <t>29/12/2025</t>
         </is>
       </c>
-      <c r="F157" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G157" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H157" s="5" t="inlineStr">
-        <is>
-          <t>59/64</t>
-        </is>
-      </c>
-      <c r="I157" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr"/>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9932,49 +9924,45 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B204" s="5" t="inlineStr">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C204" s="5" t="inlineStr">
+      <c r="C204" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D204" s="5" t="inlineStr">
+      <c r="D204" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E204" s="5" t="inlineStr">
+      <c r="E204" s="2" t="inlineStr">
         <is>
           <t>29/12/2025</t>
         </is>
       </c>
-      <c r="F204" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G204" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H204" s="5" t="inlineStr">
-        <is>
-          <t>10/62</t>
-        </is>
-      </c>
-      <c r="I204" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr"/>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -11302,49 +11290,45 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B234" s="5" t="inlineStr">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C234" s="5" t="inlineStr">
+      <c r="C234" s="2" t="inlineStr">
         <is>
           <t>CLINICAL PATHOLOGY</t>
         </is>
       </c>
-      <c r="D234" s="5" t="inlineStr">
+      <c r="D234" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E234" s="5" t="inlineStr">
+      <c r="E234" s="2" t="inlineStr">
         <is>
           <t>29/12/2025</t>
         </is>
       </c>
-      <c r="F234" s="5" t="inlineStr">
+      <c r="F234" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G234" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H234" s="5" t="inlineStr">
-        <is>
-          <t>31/60</t>
-        </is>
-      </c>
-      <c r="I234" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G234" s="2" t="inlineStr"/>
+      <c r="H234" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -11912,49 +11896,45 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B248" s="5" t="inlineStr">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C248" s="5" t="inlineStr">
+      <c r="C248" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D248" s="5" t="inlineStr">
+      <c r="D248" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E248" s="5" t="inlineStr">
+      <c r="E248" s="2" t="inlineStr">
         <is>
           <t>29/12/2025</t>
         </is>
       </c>
-      <c r="F248" s="5" t="inlineStr">
+      <c r="F248" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G248" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H248" s="5" t="inlineStr">
-        <is>
-          <t>51/60</t>
-        </is>
-      </c>
-      <c r="I248" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G248" s="2" t="inlineStr"/>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-29 03:43:00 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8">
@@ -897,49 +897,45 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>30/12/2025</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>40/66</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>0/66</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -949,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>38.1%</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1002,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>75.2%</t>
+          <t>75.7%</t>
         </is>
       </c>
     </row>
@@ -1307,22 +1303,22 @@
         <v>53</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>37.7%</t>
+          <t>35.8%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>78.0%</t>
+          <t>78.9%</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1385,22 @@
         <v>53</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>39.6%</t>
+          <t>37.7%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>82.0%</t>
+          <t>81.5%</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1467,22 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>39.6%</t>
+          <t>37.7%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>72.5%</t>
         </is>
       </c>
     </row>
@@ -1553,22 +1549,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>46.2%</t>
+          <t>44.2%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>74.4%</t>
+          <t>73.6%</t>
         </is>
       </c>
     </row>
@@ -1635,22 +1631,22 @@
         <v>54</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>37.0%</t>
+          <t>35.2%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>70.3%</t>
+          <t>72.1%</t>
         </is>
       </c>
     </row>
@@ -3953,49 +3949,45 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>30/12/2025</t>
         </is>
       </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H71" s="5" t="inlineStr">
-        <is>
-          <t>57/62</t>
-        </is>
-      </c>
-      <c r="I71" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7850,49 +7842,45 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B158" s="5" t="inlineStr">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C158" s="5" t="inlineStr">
+      <c r="C158" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D158" s="5" t="inlineStr">
+      <c r="D158" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E158" s="5" t="inlineStr">
+      <c r="E158" s="2" t="inlineStr">
         <is>
           <t>30/12/2025</t>
         </is>
       </c>
-      <c r="F158" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G158" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H158" s="5" t="inlineStr">
-        <is>
-          <t>32/64</t>
-        </is>
-      </c>
-      <c r="I158" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr"/>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9967,49 +9955,45 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B205" s="5" t="inlineStr">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C205" s="5" t="inlineStr">
+      <c r="C205" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D205" s="5" t="inlineStr">
+      <c r="D205" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E205" s="5" t="inlineStr">
+      <c r="E205" s="2" t="inlineStr">
         <is>
           <t>30/12/2025</t>
         </is>
       </c>
-      <c r="F205" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G205" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H205" s="5" t="inlineStr">
-        <is>
-          <t>58/62</t>
-        </is>
-      </c>
-      <c r="I205" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr"/>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -11939,49 +11923,45 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B249" s="5" t="inlineStr">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C249" s="5" t="inlineStr">
+      <c r="C249" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D249" s="5" t="inlineStr">
+      <c r="D249" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E249" s="5" t="inlineStr">
+      <c r="E249" s="2" t="inlineStr">
         <is>
           <t>30/12/2025</t>
         </is>
       </c>
-      <c r="F249" s="5" t="inlineStr">
+      <c r="F249" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G249" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H249" s="5" t="inlineStr">
-        <is>
-          <t>22/60</t>
-        </is>
-      </c>
-      <c r="I249" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G249" s="2" t="inlineStr"/>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-01 01:52:19 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>35.8%</t>
+          <t>34.3%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>75.9%</t>
+          <t>76.2%</t>
         </is>
       </c>
     </row>
@@ -1381,22 +1381,22 @@
         <v>53</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>35.8%</t>
+          <t>34.0%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>82.6%</t>
+          <t>83.3%</t>
         </is>
       </c>
     </row>
@@ -1463,22 +1463,22 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>35.8%</t>
+          <t>34.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>70.8%</t>
         </is>
       </c>
     </row>
@@ -1545,22 +1545,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>42.3%</t>
+          <t>40.4%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>72.7%</t>
+          <t>72.2%</t>
         </is>
       </c>
     </row>
@@ -1627,22 +1627,22 @@
         <v>54</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>31.5%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>72.1%</t>
+          <t>74.0%</t>
         </is>
       </c>
     </row>
@@ -4031,49 +4031,45 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr">
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="F73" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H73" s="5" t="inlineStr">
-        <is>
-          <t>43/62</t>
-        </is>
-      </c>
-      <c r="I73" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7920,49 +7916,45 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B160" s="5" t="inlineStr">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C160" s="5" t="inlineStr">
+      <c r="C160" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D160" s="5" t="inlineStr">
+      <c r="D160" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E160" s="5" t="inlineStr">
+      <c r="E160" s="2" t="inlineStr">
         <is>
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="F160" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G160" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H160" s="5" t="inlineStr">
-        <is>
-          <t>52/64</t>
-        </is>
-      </c>
-      <c r="I160" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr"/>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10029,49 +10021,45 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B207" s="5" t="inlineStr">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C207" s="5" t="inlineStr">
+      <c r="C207" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D207" s="5" t="inlineStr">
+      <c r="D207" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E207" s="5" t="inlineStr">
+      <c r="E207" s="2" t="inlineStr">
         <is>
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="F207" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G207" s="5" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="H207" s="5" t="inlineStr">
-        <is>
-          <t>51/62</t>
-        </is>
-      </c>
-      <c r="I207" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr"/>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -11989,49 +11977,45 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B251" s="5" t="inlineStr">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C251" s="5" t="inlineStr">
+      <c r="C251" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D251" s="5" t="inlineStr">
+      <c r="D251" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E251" s="5" t="inlineStr">
+      <c r="E251" s="2" t="inlineStr">
         <is>
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="F251" s="5" t="inlineStr">
+      <c r="F251" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G251" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H251" s="5" t="inlineStr">
-        <is>
-          <t>25/60</t>
-        </is>
-      </c>
-      <c r="I251" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G251" s="2" t="inlineStr"/>
+      <c r="H251" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I251" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-05 04:04:53 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -479,7 +479,7 @@
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="11" max="11"/>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>32.1%</t>
+          <t>30.2%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>76.1%</t>
+          <t>75.5%</t>
         </is>
       </c>
     </row>
@@ -1377,22 +1377,22 @@
         <v>53</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>32.1%</t>
+          <t>30.2%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>82.8%</t>
+          <t>82.4%</t>
         </is>
       </c>
     </row>
@@ -1459,22 +1459,22 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>32.1%</t>
+          <t>30.2%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>69.9%</t>
+          <t>68.4%</t>
         </is>
       </c>
     </row>
@@ -1541,22 +1541,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>38.5%</t>
+          <t>34.6%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>71.5%</t>
+          <t>70.5%</t>
         </is>
       </c>
     </row>
@@ -1623,22 +1623,22 @@
         <v>54</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>24.1%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>75.7%</t>
+          <t>75.1%</t>
         </is>
       </c>
     </row>
@@ -4328,49 +4328,45 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D80" s="5" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E80" s="5" t="inlineStr">
+      <c r="E80" s="2" t="inlineStr">
         <is>
           <t>05/01/2026</t>
         </is>
       </c>
-      <c r="F80" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G80" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H80" s="5" t="inlineStr">
-        <is>
-          <t>56/62</t>
-        </is>
-      </c>
-      <c r="I80" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7356,49 +7352,45 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B148" s="5" t="inlineStr">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C148" s="5" t="inlineStr">
+      <c r="C148" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D148" s="5" t="inlineStr">
+      <c r="D148" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E148" s="5" t="inlineStr">
+      <c r="E148" s="2" t="inlineStr">
         <is>
           <t>05/01/2026</t>
         </is>
       </c>
-      <c r="F148" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G148" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H148" s="5" t="inlineStr">
-        <is>
-          <t>60/64</t>
-        </is>
-      </c>
-      <c r="I148" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr"/>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -8796,49 +8788,45 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B180" s="5" t="inlineStr">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C180" s="5" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>CLINICAL PATHOLOGY</t>
         </is>
       </c>
-      <c r="D180" s="5" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E180" s="5" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>05/01/2026</t>
         </is>
       </c>
-      <c r="F180" s="5" t="inlineStr">
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G180" s="5" t="inlineStr">
-        <is>
-          <t>2026/2027, 2027/2028</t>
-        </is>
-      </c>
-      <c r="H180" s="5" t="inlineStr">
-        <is>
-          <t>43/62</t>
-        </is>
-      </c>
-      <c r="I180" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G180" s="2" t="inlineStr"/>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9242,49 +9230,45 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B190" s="5" t="inlineStr">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C190" s="5" t="inlineStr">
+      <c r="C190" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D190" s="5" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E190" s="5" t="inlineStr">
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>05/01/2026</t>
         </is>
       </c>
-      <c r="F190" s="5" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G190" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H190" s="5" t="inlineStr">
-        <is>
-          <t>57/62</t>
-        </is>
-      </c>
-      <c r="I190" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G190" s="2" t="inlineStr"/>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10349,49 +10333,45 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B215" s="5" t="inlineStr">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C215" s="5" t="inlineStr">
+      <c r="C215" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D215" s="5" t="inlineStr">
+      <c r="D215" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E215" s="5" t="inlineStr">
+      <c r="E215" s="2" t="inlineStr">
         <is>
           <t>05/01/2026</t>
         </is>
       </c>
-      <c r="F215" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G215" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H215" s="5" t="inlineStr">
-        <is>
-          <t>50/60</t>
-        </is>
-      </c>
-      <c r="I215" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr"/>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 01:15:51 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>24.9%</t>
+          <t>23.0%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>74.4%</t>
+          <t>73.3%</t>
         </is>
       </c>
     </row>
@@ -1283,69 +1283,65 @@
         <v>53</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>24.5%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>81.6%</t>
+          <t>81.1%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>58/66</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>0/66</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
@@ -1365,22 +1361,22 @@
         <v>53</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>24.5%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>82.0%</t>
+          <t>80.9%</t>
         </is>
       </c>
     </row>
@@ -1447,22 +1443,22 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>24.5%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>66.2%</t>
+          <t>64.6%</t>
         </is>
       </c>
     </row>
@@ -1529,22 +1525,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>67.7%</t>
+          <t>65.5%</t>
         </is>
       </c>
     </row>
@@ -5384,49 +5380,45 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B104" s="5" t="inlineStr">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D104" s="5" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E104" s="5" t="inlineStr">
+      <c r="E104" s="2" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
       </c>
-      <c r="F104" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G104" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H104" s="5" t="inlineStr">
-        <is>
-          <t>59/62</t>
-        </is>
-      </c>
-      <c r="I104" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7500,49 +7492,45 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B152" s="5" t="inlineStr">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C152" s="5" t="inlineStr">
+      <c r="C152" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D152" s="5" t="inlineStr">
+      <c r="D152" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E152" s="5" t="inlineStr">
+      <c r="E152" s="2" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
       </c>
-      <c r="F152" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G152" s="5" t="inlineStr">
-        <is>
-          <t>2027/2028</t>
-        </is>
-      </c>
-      <c r="H152" s="5" t="inlineStr">
-        <is>
-          <t>55/64</t>
-        </is>
-      </c>
-      <c r="I152" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr"/>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -8795,49 +8783,45 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B181" s="5" t="inlineStr">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C181" s="5" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t>CLINICAL PATHOLOGY</t>
         </is>
       </c>
-      <c r="D181" s="5" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E181" s="5" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
       </c>
-      <c r="F181" s="5" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G181" s="5" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="H181" s="5" t="inlineStr">
-        <is>
-          <t>46/62</t>
-        </is>
-      </c>
-      <c r="I181" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G181" s="2" t="inlineStr"/>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9366,49 +9350,45 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B194" s="5" t="inlineStr">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C194" s="5" t="inlineStr">
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D194" s="5" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E194" s="5" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
       </c>
-      <c r="F194" s="5" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G194" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H194" s="5" t="inlineStr">
-        <is>
-          <t>56/62</t>
-        </is>
-      </c>
-      <c r="I194" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G194" s="2" t="inlineStr"/>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-13 01:13:40 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>21.1%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>73.3%</t>
+          <t>72.2%</t>
         </is>
       </c>
     </row>
@@ -1283,22 +1283,22 @@
         <v>53</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>24.5%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>81.1%</t>
+          <t>79.8%</t>
         </is>
       </c>
     </row>
@@ -1361,69 +1361,65 @@
         <v>53</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>20.8%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>80.9%</t>
+          <t>80.4%</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>64/66</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>0/66</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -1443,22 +1439,22 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>20.8%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>64.6%</t>
+          <t>62.6%</t>
         </is>
       </c>
     </row>
@@ -1525,22 +1521,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>65.5%</t>
+          <t>64.7%</t>
         </is>
       </c>
     </row>
@@ -1607,22 +1603,22 @@
         <v>54</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>74.7%</t>
+          <t>73.8%</t>
         </is>
       </c>
     </row>
@@ -5423,49 +5419,45 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C105" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D105" s="5" t="inlineStr">
+      <c r="D105" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E105" s="5" t="inlineStr">
+      <c r="E105" s="2" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
       </c>
-      <c r="F105" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G105" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H105" s="5" t="inlineStr">
-        <is>
-          <t>54/62</t>
-        </is>
-      </c>
-      <c r="I105" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr"/>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7535,49 +7527,45 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B153" s="5" t="inlineStr">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C153" s="5" t="inlineStr">
+      <c r="C153" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D153" s="5" t="inlineStr">
+      <c r="D153" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E153" s="5" t="inlineStr">
+      <c r="E153" s="2" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
       </c>
-      <c r="F153" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G153" s="5" t="inlineStr">
-        <is>
-          <t>2027/2028</t>
-        </is>
-      </c>
-      <c r="H153" s="5" t="inlineStr">
-        <is>
-          <t>55/64</t>
-        </is>
-      </c>
-      <c r="I153" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr"/>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9393,49 +9381,45 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B195" s="5" t="inlineStr">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C195" s="5" t="inlineStr">
+      <c r="C195" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D195" s="5" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E195" s="5" t="inlineStr">
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
       </c>
-      <c r="F195" s="5" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G195" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H195" s="5" t="inlineStr">
-        <is>
-          <t>47/62</t>
-        </is>
-      </c>
-      <c r="I195" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G195" s="2" t="inlineStr"/>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10480,49 +10464,45 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B220" s="5" t="inlineStr">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C220" s="5" t="inlineStr">
+      <c r="C220" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D220" s="5" t="inlineStr">
+      <c r="D220" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E220" s="5" t="inlineStr">
+      <c r="E220" s="2" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
       </c>
-      <c r="F220" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G220" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H220" s="5" t="inlineStr">
-        <is>
-          <t>50/60</t>
-        </is>
-      </c>
-      <c r="I220" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr"/>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-14 01:05:44 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>72.2%</t>
+          <t>73.1%</t>
         </is>
       </c>
     </row>
@@ -1283,22 +1283,22 @@
         <v>53</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>20.8%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>79.8%</t>
+          <t>83.2%</t>
         </is>
       </c>
     </row>
@@ -1361,22 +1361,22 @@
         <v>53</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>80.4%</t>
+          <t>78.7%</t>
         </is>
       </c>
     </row>
@@ -1439,69 +1439,65 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>62.6%</t>
+          <t>61.9%</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>28/66</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>0/66</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
@@ -1521,22 +1517,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>64.7%</t>
+          <t>65.3%</t>
         </is>
       </c>
     </row>
@@ -1603,22 +1599,22 @@
         <v>54</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>73.8%</t>
+          <t>75.6%</t>
         </is>
       </c>
     </row>
@@ -5462,49 +5458,45 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B106" s="5" t="inlineStr">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
+      <c r="C106" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D106" s="5" t="inlineStr">
+      <c r="D106" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E106" s="5" t="inlineStr">
+      <c r="E106" s="2" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
       </c>
-      <c r="F106" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G106" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H106" s="5" t="inlineStr">
-        <is>
-          <t>60/62</t>
-        </is>
-      </c>
-      <c r="I106" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr"/>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7570,49 +7562,45 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B154" s="5" t="inlineStr">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C154" s="5" t="inlineStr">
+      <c r="C154" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D154" s="5" t="inlineStr">
+      <c r="D154" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E154" s="5" t="inlineStr">
+      <c r="E154" s="2" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
       </c>
-      <c r="F154" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G154" s="5" t="inlineStr">
-        <is>
-          <t>2027/2028</t>
-        </is>
-      </c>
-      <c r="H154" s="5" t="inlineStr">
-        <is>
-          <t>45/64</t>
-        </is>
-      </c>
-      <c r="I154" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr"/>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -8814,49 +8802,45 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B182" s="5" t="inlineStr">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C182" s="5" t="inlineStr">
+      <c r="C182" s="2" t="inlineStr">
         <is>
           <t>CLINICAL PATHOLOGY</t>
         </is>
       </c>
-      <c r="D182" s="5" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E182" s="5" t="inlineStr">
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
       </c>
-      <c r="F182" s="5" t="inlineStr">
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G182" s="5" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="H182" s="5" t="inlineStr">
-        <is>
-          <t>34/62</t>
-        </is>
-      </c>
-      <c r="I182" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G182" s="2" t="inlineStr"/>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9424,49 +9408,45 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B196" s="5" t="inlineStr">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C196" s="5" t="inlineStr">
+      <c r="C196" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D196" s="5" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E196" s="5" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
       </c>
-      <c r="F196" s="5" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G196" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H196" s="5" t="inlineStr">
-        <is>
-          <t>42/62</t>
-        </is>
-      </c>
-      <c r="I196" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G196" s="2" t="inlineStr"/>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10507,49 +10487,45 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B221" s="5" t="inlineStr">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C221" s="5" t="inlineStr">
+      <c r="C221" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D221" s="5" t="inlineStr">
+      <c r="D221" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E221" s="5" t="inlineStr">
+      <c r="E221" s="2" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
       </c>
-      <c r="F221" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G221" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H221" s="5" t="inlineStr">
-        <is>
-          <t>35/60</t>
-        </is>
-      </c>
-      <c r="I221" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr"/>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 01:12:08 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>74.6%</t>
+          <t>74.2%</t>
         </is>
       </c>
     </row>
@@ -1517,22 +1517,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>62.7%</t>
+          <t>59.0%</t>
         </is>
       </c>
     </row>
@@ -8039,49 +8039,45 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B165" s="6" t="inlineStr">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C165" s="6" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D165" s="6" t="inlineStr">
+      <c r="D165" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E165" s="6" t="inlineStr">
+      <c r="E165" s="2" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
       </c>
-      <c r="F165" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G165" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H165" s="6" t="inlineStr">
-        <is>
-          <t>55/62</t>
-        </is>
-      </c>
-      <c r="I165" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr"/>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-18 01:02:24 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -96,10 +96,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>74.2%</t>
+          <t>73.1%</t>
         </is>
       </c>
     </row>
@@ -1283,22 +1283,22 @@
         <v>53</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>86.8%</t>
+          <t>86.0%</t>
         </is>
       </c>
     </row>
@@ -1361,22 +1361,22 @@
         <v>53</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>81.0%</t>
+          <t>80.6%</t>
         </is>
       </c>
     </row>
@@ -1439,22 +1439,22 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>64.1%</t>
+          <t>61.7%</t>
         </is>
       </c>
     </row>
@@ -1517,22 +1517,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>54.3%</t>
         </is>
       </c>
     </row>
@@ -1595,22 +1595,22 @@
         <v>54</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>75.6%</t>
+          <t>76.7%</t>
         </is>
       </c>
     </row>
@@ -1865,265 +1865,261 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>0/66</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>Session missed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>B2A</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>DERMATOLOGY</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>19/01/2026</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>62/66</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>55/66</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
-        </is>
-      </c>
-      <c r="L25" s="7" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="M25" s="4" t="inlineStr">
-        <is>
-          <t>Session missed</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>Future session</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>19/01/2026</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>20/01/2026</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>55/66</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>59/66</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L26" s="8" t="inlineStr">
-        <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="M26" s="4" t="inlineStr">
-        <is>
-          <t>Future session</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>20/01/2026</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>21/01/2026</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>59/66</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>65/66</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>21/01/2026</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>22/01/2026</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>65/66</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>B2A</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>DERMATOLOGY</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>22/01/2026</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>65/66</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -2990,235 +2986,235 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>08/02/2026</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>55/66</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
+      <c r="I50" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="7" t="inlineStr">
         <is>
           <t>09/02/2026</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H51" s="7" t="inlineStr">
         <is>
           <t>58/66</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
+      <c r="I51" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E52" s="7" t="inlineStr">
         <is>
           <t>10/02/2026</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>33/66</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
+      <c r="I52" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E53" s="7" t="inlineStr">
         <is>
           <t>11/02/2026</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="H53" s="7" t="inlineStr">
         <is>
           <t>60/66</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
+      <c r="I53" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
         <is>
           <t>12/02/2026</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H54" s="7" t="inlineStr">
         <is>
           <t>61/66</t>
         </is>
       </c>
-      <c r="I54" s="6" t="inlineStr">
+      <c r="I54" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -4859,329 +4855,325 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C93" s="6" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D93" s="6" t="inlineStr">
+      <c r="D93" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E93" s="6" t="inlineStr">
+      <c r="E93" s="2" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
       </c>
-      <c r="F93" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G93" s="6" t="inlineStr">
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>PSYCHIATRY</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>19/01/2026</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>2027/2028</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>48/62</t>
+        </is>
+      </c>
+      <c r="I94" s="7" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>PSYCHIATRY</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>20/01/2026</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H93" s="6" t="inlineStr">
-        <is>
-          <t>52/62</t>
-        </is>
-      </c>
-      <c r="I93" s="6" t="inlineStr">
+      <c r="H95" s="7" t="inlineStr">
+        <is>
+          <t>58/62</t>
+        </is>
+      </c>
+      <c r="I95" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B94" s="6" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C94" s="6" t="inlineStr">
+      <c r="C96" s="7" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D94" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E94" s="6" t="inlineStr">
-        <is>
-          <t>19/01/2026</t>
-        </is>
-      </c>
-      <c r="F94" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G94" s="6" t="inlineStr">
-        <is>
-          <t>2027/2028</t>
-        </is>
-      </c>
-      <c r="H94" s="6" t="inlineStr">
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>21/01/2026</t>
+        </is>
+      </c>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G96" s="7" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H96" s="7" t="inlineStr">
+        <is>
+          <t>57/62</t>
+        </is>
+      </c>
+      <c r="I96" s="7" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>PSYCHIATRY</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>22/01/2026</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H97" s="7" t="inlineStr">
+        <is>
+          <t>44/62</t>
+        </is>
+      </c>
+      <c r="I97" s="7" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>PSYCHIATRY</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>08/02/2026</t>
+        </is>
+      </c>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H98" s="7" t="inlineStr">
+        <is>
+          <t>49/62</t>
+        </is>
+      </c>
+      <c r="I98" s="7" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>PSYCHIATRY</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H99" s="7" t="inlineStr">
         <is>
           <t>48/62</t>
         </is>
       </c>
-      <c r="I94" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="inlineStr">
-        <is>
-          <t>PSYCHIATRY</t>
-        </is>
-      </c>
-      <c r="D95" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E95" s="6" t="inlineStr">
-        <is>
-          <t>20/01/2026</t>
-        </is>
-      </c>
-      <c r="F95" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G95" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H95" s="6" t="inlineStr">
-        <is>
-          <t>58/62</t>
-        </is>
-      </c>
-      <c r="I95" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>PSYCHIATRY</t>
-        </is>
-      </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E96" s="6" t="inlineStr">
-        <is>
-          <t>21/01/2026</t>
-        </is>
-      </c>
-      <c r="F96" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G96" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H96" s="6" t="inlineStr">
-        <is>
-          <t>57/62</t>
-        </is>
-      </c>
-      <c r="I96" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t>PSYCHIATRY</t>
-        </is>
-      </c>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E97" s="6" t="inlineStr">
-        <is>
-          <t>22/01/2026</t>
-        </is>
-      </c>
-      <c r="F97" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G97" s="6" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="H97" s="6" t="inlineStr">
-        <is>
-          <t>44/62</t>
-        </is>
-      </c>
-      <c r="I97" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>PSYCHIATRY</t>
-        </is>
-      </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E98" s="6" t="inlineStr">
-        <is>
-          <t>08/02/2026</t>
-        </is>
-      </c>
-      <c r="F98" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G98" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H98" s="6" t="inlineStr">
-        <is>
-          <t>49/62</t>
-        </is>
-      </c>
-      <c r="I98" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B99" s="6" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr">
-        <is>
-          <t>PSYCHIATRY</t>
-        </is>
-      </c>
-      <c r="D99" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E99" s="6" t="inlineStr">
-        <is>
-          <t>09/02/2026</t>
-        </is>
-      </c>
-      <c r="F99" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G99" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H99" s="6" t="inlineStr">
-        <is>
-          <t>48/62</t>
-        </is>
-      </c>
-      <c r="I99" s="6" t="inlineStr">
+      <c r="I99" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -5231,94 +5223,94 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C101" s="6" t="inlineStr">
+      <c r="C101" s="7" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D101" s="6" t="inlineStr">
+      <c r="D101" s="7" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E101" s="6" t="inlineStr">
+      <c r="E101" s="7" t="inlineStr">
         <is>
           <t>11/02/2026</t>
         </is>
       </c>
-      <c r="F101" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G101" s="6" t="inlineStr">
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G101" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H101" s="6" t="inlineStr">
+      <c r="H101" s="7" t="inlineStr">
         <is>
           <t>40/62</t>
         </is>
       </c>
-      <c r="I101" s="6" t="inlineStr">
+      <c r="I101" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B102" s="6" t="inlineStr">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B102" s="7" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C102" s="6" t="inlineStr">
+      <c r="C102" s="7" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D102" s="6" t="inlineStr">
+      <c r="D102" s="7" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E102" s="6" t="inlineStr">
+      <c r="E102" s="7" t="inlineStr">
         <is>
           <t>12/02/2026</t>
         </is>
       </c>
-      <c r="F102" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G102" s="6" t="inlineStr">
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G102" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H102" s="6" t="inlineStr">
+      <c r="H102" s="7" t="inlineStr">
         <is>
           <t>56/62</t>
         </is>
       </c>
-      <c r="I102" s="6" t="inlineStr">
+      <c r="I102" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -6400,47 +6392,47 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B128" s="6" t="inlineStr">
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B128" s="7" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C128" s="6" t="inlineStr">
+      <c r="C128" s="7" t="inlineStr">
         <is>
           <t>CLINICAL PATHOLOGY</t>
         </is>
       </c>
-      <c r="D128" s="6" t="inlineStr">
+      <c r="D128" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E128" s="6" t="inlineStr">
+      <c r="E128" s="7" t="inlineStr">
         <is>
           <t>21/01/2026</t>
         </is>
       </c>
-      <c r="F128" s="6" t="inlineStr">
+      <c r="F128" s="7" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G128" s="6" t="inlineStr">
+      <c r="G128" s="7" t="inlineStr">
         <is>
           <t>2027/2028</t>
         </is>
       </c>
-      <c r="H128" s="6" t="inlineStr">
+      <c r="H128" s="7" t="inlineStr">
         <is>
           <t>29/64</t>
         </is>
       </c>
-      <c r="I128" s="6" t="inlineStr">
+      <c r="I128" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -6791,376 +6783,372 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B137" s="6" t="inlineStr">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C137" s="6" t="inlineStr">
+      <c r="C137" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D137" s="6" t="inlineStr">
+      <c r="D137" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E137" s="6" t="inlineStr">
+      <c r="E137" s="2" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
       </c>
-      <c r="F137" s="6" t="inlineStr">
+      <c r="F137" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G137" s="6" t="inlineStr">
+      <c r="G137" s="2" t="inlineStr"/>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B138" s="7" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+      <c r="C138" s="7" t="inlineStr">
+        <is>
+          <t>IMMUNOLOGY/HAEMATOLOGY</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E138" s="7" t="inlineStr">
+        <is>
+          <t>19/01/2026</t>
+        </is>
+      </c>
+      <c r="F138" s="7" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G138" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H137" s="6" t="inlineStr">
+      <c r="H138" s="7" t="inlineStr">
+        <is>
+          <t>60/64</t>
+        </is>
+      </c>
+      <c r="I138" s="7" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
+      <c r="C139" s="7" t="inlineStr">
+        <is>
+          <t>IMMUNOLOGY/HAEMATOLOGY</t>
+        </is>
+      </c>
+      <c r="D139" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E139" s="7" t="inlineStr">
+        <is>
+          <t>20/01/2026</t>
+        </is>
+      </c>
+      <c r="F139" s="7" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G139" s="7" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H139" s="7" t="inlineStr">
         <is>
           <t>53/64</t>
         </is>
       </c>
-      <c r="I137" s="6" t="inlineStr">
+      <c r="I139" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B138" s="6" t="inlineStr">
+    <row r="140">
+      <c r="A140" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B140" s="7" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C138" s="6" t="inlineStr">
+      <c r="C140" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D138" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E138" s="6" t="inlineStr">
-        <is>
-          <t>19/01/2026</t>
-        </is>
-      </c>
-      <c r="F138" s="6" t="inlineStr">
+      <c r="D140" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E140" s="7" t="inlineStr">
+        <is>
+          <t>21/01/2026</t>
+        </is>
+      </c>
+      <c r="F140" s="7" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G138" s="6" t="inlineStr">
+      <c r="G140" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H138" s="6" t="inlineStr">
-        <is>
-          <t>60/64</t>
-        </is>
-      </c>
-      <c r="I138" s="6" t="inlineStr">
+      <c r="H140" s="7" t="inlineStr">
+        <is>
+          <t>54/64</t>
+        </is>
+      </c>
+      <c r="I140" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B139" s="6" t="inlineStr">
+    <row r="141">
+      <c r="A141" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C139" s="6" t="inlineStr">
+      <c r="C141" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D139" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E139" s="6" t="inlineStr">
-        <is>
-          <t>20/01/2026</t>
-        </is>
-      </c>
-      <c r="F139" s="6" t="inlineStr">
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E141" s="7" t="inlineStr">
+        <is>
+          <t>22/01/2026</t>
+        </is>
+      </c>
+      <c r="F141" s="7" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G139" s="6" t="inlineStr">
+      <c r="G141" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H139" s="6" t="inlineStr">
-        <is>
-          <t>53/64</t>
-        </is>
-      </c>
-      <c r="I139" s="6" t="inlineStr">
+      <c r="H141" s="7" t="inlineStr">
+        <is>
+          <t>34/64</t>
+        </is>
+      </c>
+      <c r="I141" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B140" s="6" t="inlineStr">
+    <row r="142">
+      <c r="A142" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B142" s="7" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C140" s="6" t="inlineStr">
+      <c r="C142" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D140" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E140" s="6" t="inlineStr">
-        <is>
-          <t>21/01/2026</t>
-        </is>
-      </c>
-      <c r="F140" s="6" t="inlineStr">
+      <c r="D142" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E142" s="7" t="inlineStr">
+        <is>
+          <t>08/02/2026</t>
+        </is>
+      </c>
+      <c r="F142" s="7" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G140" s="6" t="inlineStr">
+      <c r="G142" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H140" s="6" t="inlineStr">
-        <is>
-          <t>54/64</t>
-        </is>
-      </c>
-      <c r="I140" s="6" t="inlineStr">
+      <c r="H142" s="7" t="inlineStr">
+        <is>
+          <t>36/64</t>
+        </is>
+      </c>
+      <c r="I142" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B141" s="6" t="inlineStr">
+    <row r="143">
+      <c r="A143" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C141" s="6" t="inlineStr">
+      <c r="C143" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D141" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E141" s="6" t="inlineStr">
-        <is>
-          <t>22/01/2026</t>
-        </is>
-      </c>
-      <c r="F141" s="6" t="inlineStr">
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="F143" s="7" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G141" s="6" t="inlineStr">
+      <c r="G143" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H141" s="6" t="inlineStr">
-        <is>
-          <t>34/64</t>
-        </is>
-      </c>
-      <c r="I141" s="6" t="inlineStr">
+      <c r="H143" s="7" t="inlineStr">
+        <is>
+          <t>24/64</t>
+        </is>
+      </c>
+      <c r="I143" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B142" s="6" t="inlineStr">
+    <row r="144">
+      <c r="A144" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B144" s="7" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C142" s="6" t="inlineStr">
+      <c r="C144" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D142" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E142" s="6" t="inlineStr">
-        <is>
-          <t>08/02/2026</t>
-        </is>
-      </c>
-      <c r="F142" s="6" t="inlineStr">
+      <c r="D144" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>10/02/2026</t>
+        </is>
+      </c>
+      <c r="F144" s="7" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G142" s="6" t="inlineStr">
+      <c r="G144" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H142" s="6" t="inlineStr">
-        <is>
-          <t>36/64</t>
-        </is>
-      </c>
-      <c r="I142" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B143" s="6" t="inlineStr">
-        <is>
-          <t>B2C</t>
-        </is>
-      </c>
-      <c r="C143" s="6" t="inlineStr">
-        <is>
-          <t>IMMUNOLOGY/HAEMATOLOGY</t>
-        </is>
-      </c>
-      <c r="D143" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E143" s="6" t="inlineStr">
-        <is>
-          <t>09/02/2026</t>
-        </is>
-      </c>
-      <c r="F143" s="6" t="inlineStr">
-        <is>
-          <t>10:00:00</t>
-        </is>
-      </c>
-      <c r="G143" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H143" s="6" t="inlineStr">
-        <is>
-          <t>24/64</t>
-        </is>
-      </c>
-      <c r="I143" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B144" s="6" t="inlineStr">
-        <is>
-          <t>B2C</t>
-        </is>
-      </c>
-      <c r="C144" s="6" t="inlineStr">
-        <is>
-          <t>IMMUNOLOGY/HAEMATOLOGY</t>
-        </is>
-      </c>
-      <c r="D144" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E144" s="6" t="inlineStr">
-        <is>
-          <t>10/02/2026</t>
-        </is>
-      </c>
-      <c r="F144" s="6" t="inlineStr">
-        <is>
-          <t>10:00:00</t>
-        </is>
-      </c>
-      <c r="G144" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H144" s="6" t="inlineStr">
+      <c r="H144" s="7" t="inlineStr">
         <is>
           <t>26/64</t>
         </is>
       </c>
-      <c r="I144" s="6" t="inlineStr">
+      <c r="I144" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -7855,141 +7843,141 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B161" s="6" t="inlineStr">
+      <c r="A161" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B161" s="7" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C161" s="6" t="inlineStr">
+      <c r="C161" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D161" s="6" t="inlineStr">
+      <c r="D161" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E161" s="6" t="inlineStr">
+      <c r="E161" s="7" t="inlineStr">
         <is>
           <t>07/02/2026</t>
         </is>
       </c>
-      <c r="F161" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G161" s="6" t="inlineStr">
+      <c r="F161" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G161" s="7" t="inlineStr">
         <is>
           <t>2024/2025</t>
         </is>
       </c>
-      <c r="H161" s="6" t="inlineStr">
+      <c r="H161" s="7" t="inlineStr">
         <is>
           <t>43/62</t>
         </is>
       </c>
-      <c r="I161" s="6" t="inlineStr">
+      <c r="I161" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B162" s="6" t="inlineStr">
+      <c r="A162" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B162" s="7" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C162" s="6" t="inlineStr">
+      <c r="C162" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D162" s="6" t="inlineStr">
+      <c r="D162" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E162" s="6" t="inlineStr">
+      <c r="E162" s="7" t="inlineStr">
         <is>
           <t>08/02/2026</t>
         </is>
       </c>
-      <c r="F162" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G162" s="6" t="inlineStr">
+      <c r="F162" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G162" s="7" t="inlineStr">
         <is>
           <t>2024/2025</t>
         </is>
       </c>
-      <c r="H162" s="6" t="inlineStr">
+      <c r="H162" s="7" t="inlineStr">
         <is>
           <t>24/62</t>
         </is>
       </c>
-      <c r="I162" s="6" t="inlineStr">
+      <c r="I162" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B163" s="6" t="inlineStr">
+      <c r="A163" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B163" s="7" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C163" s="6" t="inlineStr">
+      <c r="C163" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D163" s="6" t="inlineStr">
+      <c r="D163" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E163" s="6" t="inlineStr">
+      <c r="E163" s="7" t="inlineStr">
         <is>
           <t>09/02/2026</t>
         </is>
       </c>
-      <c r="F163" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G163" s="6" t="inlineStr">
+      <c r="F163" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G163" s="7" t="inlineStr">
         <is>
           <t>2024/2025</t>
         </is>
       </c>
-      <c r="H163" s="6" t="inlineStr">
+      <c r="H163" s="7" t="inlineStr">
         <is>
           <t>23/62</t>
         </is>
       </c>
-      <c r="I163" s="6" t="inlineStr">
+      <c r="I163" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -8082,188 +8070,184 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B166" s="6" t="inlineStr">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C166" s="6" t="inlineStr">
+      <c r="C166" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D166" s="6" t="inlineStr">
+      <c r="D166" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E166" s="6" t="inlineStr">
+      <c r="E166" s="2" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
       </c>
-      <c r="F166" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G166" s="6" t="inlineStr">
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr"/>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B167" s="7" t="inlineStr">
+        <is>
+          <t>B2D</t>
+        </is>
+      </c>
+      <c r="C167" s="7" t="inlineStr">
+        <is>
+          <t>CARDIOLOGY</t>
+        </is>
+      </c>
+      <c r="D167" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E167" s="7" t="inlineStr">
+        <is>
+          <t>19/01/2026</t>
+        </is>
+      </c>
+      <c r="F167" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G167" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H166" s="6" t="inlineStr">
-        <is>
-          <t>54/62</t>
-        </is>
-      </c>
-      <c r="I166" s="6" t="inlineStr">
+      <c r="H167" s="7" t="inlineStr">
+        <is>
+          <t>49/62</t>
+        </is>
+      </c>
+      <c r="I167" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="167">
-      <c r="A167" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B167" s="6" t="inlineStr">
+    <row r="168">
+      <c r="A168" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B168" s="7" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C167" s="6" t="inlineStr">
+      <c r="C168" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D167" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E167" s="6" t="inlineStr">
-        <is>
-          <t>19/01/2026</t>
-        </is>
-      </c>
-      <c r="F167" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G167" s="6" t="inlineStr">
+      <c r="D168" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E168" s="7" t="inlineStr">
+        <is>
+          <t>20/01/2026</t>
+        </is>
+      </c>
+      <c r="F168" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G168" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H167" s="6" t="inlineStr">
-        <is>
-          <t>49/62</t>
-        </is>
-      </c>
-      <c r="I167" s="6" t="inlineStr">
+      <c r="H168" s="7" t="inlineStr">
+        <is>
+          <t>11/62</t>
+        </is>
+      </c>
+      <c r="I168" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="168">
-      <c r="A168" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B168" s="6" t="inlineStr">
+    <row r="169">
+      <c r="A169" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B169" s="7" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C168" s="6" t="inlineStr">
+      <c r="C169" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D168" s="6" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E168" s="6" t="inlineStr">
-        <is>
-          <t>20/01/2026</t>
-        </is>
-      </c>
-      <c r="F168" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G168" s="6" t="inlineStr">
+      <c r="D169" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E169" s="7" t="inlineStr">
+        <is>
+          <t>21/01/2026</t>
+        </is>
+      </c>
+      <c r="F169" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G169" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H168" s="6" t="inlineStr">
-        <is>
-          <t>11/62</t>
-        </is>
-      </c>
-      <c r="I168" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B169" s="6" t="inlineStr">
-        <is>
-          <t>B2D</t>
-        </is>
-      </c>
-      <c r="C169" s="6" t="inlineStr">
-        <is>
-          <t>CARDIOLOGY</t>
-        </is>
-      </c>
-      <c r="D169" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E169" s="6" t="inlineStr">
-        <is>
-          <t>21/01/2026</t>
-        </is>
-      </c>
-      <c r="F169" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G169" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H169" s="6" t="inlineStr">
+      <c r="H169" s="7" t="inlineStr">
         <is>
           <t>52/62</t>
         </is>
       </c>
-      <c r="I169" s="6" t="inlineStr">
+      <c r="I169" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -10506,423 +10490,419 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B222" s="6" t="inlineStr">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C222" s="6" t="inlineStr">
+      <c r="C222" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D222" s="6" t="inlineStr">
+      <c r="D222" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E222" s="6" t="inlineStr">
+      <c r="E222" s="2" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
       </c>
-      <c r="F222" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G222" s="6" t="inlineStr">
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr"/>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B223" s="7" t="inlineStr">
+        <is>
+          <t>B2E</t>
+        </is>
+      </c>
+      <c r="C223" s="7" t="inlineStr">
+        <is>
+          <t>CHEST</t>
+        </is>
+      </c>
+      <c r="D223" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E223" s="7" t="inlineStr">
+        <is>
+          <t>19/01/2026</t>
+        </is>
+      </c>
+      <c r="F223" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G223" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H222" s="6" t="inlineStr">
-        <is>
-          <t>40/60</t>
-        </is>
-      </c>
-      <c r="I222" s="6" t="inlineStr">
+      <c r="H223" s="7" t="inlineStr">
+        <is>
+          <t>49/60</t>
+        </is>
+      </c>
+      <c r="I223" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="223">
-      <c r="A223" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B223" s="6" t="inlineStr">
+    <row r="224">
+      <c r="A224" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B224" s="7" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C223" s="6" t="inlineStr">
+      <c r="C224" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D223" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E223" s="6" t="inlineStr">
-        <is>
-          <t>19/01/2026</t>
-        </is>
-      </c>
-      <c r="F223" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G223" s="6" t="inlineStr">
+      <c r="D224" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E224" s="7" t="inlineStr">
+        <is>
+          <t>20/01/2026</t>
+        </is>
+      </c>
+      <c r="F224" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G224" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H223" s="6" t="inlineStr">
-        <is>
-          <t>49/60</t>
-        </is>
-      </c>
-      <c r="I223" s="6" t="inlineStr">
+      <c r="H224" s="7" t="inlineStr">
+        <is>
+          <t>54/60</t>
+        </is>
+      </c>
+      <c r="I224" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="224">
-      <c r="A224" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B224" s="6" t="inlineStr">
+    <row r="225">
+      <c r="A225" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B225" s="7" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C224" s="6" t="inlineStr">
+      <c r="C225" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D224" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E224" s="6" t="inlineStr">
-        <is>
-          <t>20/01/2026</t>
-        </is>
-      </c>
-      <c r="F224" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G224" s="6" t="inlineStr">
+      <c r="D225" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E225" s="7" t="inlineStr">
+        <is>
+          <t>21/01/2026</t>
+        </is>
+      </c>
+      <c r="F225" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G225" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H224" s="6" t="inlineStr">
+      <c r="H225" s="7" t="inlineStr">
         <is>
           <t>54/60</t>
         </is>
       </c>
-      <c r="I224" s="6" t="inlineStr">
+      <c r="I225" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="225">
-      <c r="A225" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B225" s="6" t="inlineStr">
+    <row r="226">
+      <c r="A226" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B226" s="7" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C225" s="6" t="inlineStr">
+      <c r="C226" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D225" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E225" s="6" t="inlineStr">
-        <is>
-          <t>21/01/2026</t>
-        </is>
-      </c>
-      <c r="F225" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G225" s="6" t="inlineStr">
+      <c r="D226" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E226" s="7" t="inlineStr">
+        <is>
+          <t>22/01/2026</t>
+        </is>
+      </c>
+      <c r="F226" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G226" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H225" s="6" t="inlineStr">
-        <is>
-          <t>54/60</t>
-        </is>
-      </c>
-      <c r="I225" s="6" t="inlineStr">
+      <c r="H226" s="7" t="inlineStr">
+        <is>
+          <t>35/60</t>
+        </is>
+      </c>
+      <c r="I226" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="226">
-      <c r="A226" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B226" s="6" t="inlineStr">
+    <row r="227">
+      <c r="A227" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B227" s="7" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C226" s="6" t="inlineStr">
+      <c r="C227" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D226" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E226" s="6" t="inlineStr">
-        <is>
-          <t>22/01/2026</t>
-        </is>
-      </c>
-      <c r="F226" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G226" s="6" t="inlineStr">
+      <c r="D227" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E227" s="7" t="inlineStr">
+        <is>
+          <t>08/02/2026</t>
+        </is>
+      </c>
+      <c r="F227" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G227" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H226" s="6" t="inlineStr">
-        <is>
-          <t>35/60</t>
-        </is>
-      </c>
-      <c r="I226" s="6" t="inlineStr">
+      <c r="H227" s="7" t="inlineStr">
+        <is>
+          <t>45/60</t>
+        </is>
+      </c>
+      <c r="I227" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B227" s="6" t="inlineStr">
+    <row r="228">
+      <c r="A228" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B228" s="7" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C227" s="6" t="inlineStr">
+      <c r="C228" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D227" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E227" s="6" t="inlineStr">
-        <is>
-          <t>08/02/2026</t>
-        </is>
-      </c>
-      <c r="F227" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G227" s="6" t="inlineStr">
+      <c r="D228" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E228" s="7" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="F228" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G228" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H227" s="6" t="inlineStr">
-        <is>
-          <t>45/60</t>
-        </is>
-      </c>
-      <c r="I227" s="6" t="inlineStr">
+      <c r="H228" s="7" t="inlineStr">
+        <is>
+          <t>43/60</t>
+        </is>
+      </c>
+      <c r="I228" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
     </row>
-    <row r="228">
-      <c r="A228" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B228" s="6" t="inlineStr">
+    <row r="229">
+      <c r="A229" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B229" s="7" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C228" s="6" t="inlineStr">
+      <c r="C229" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D228" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E228" s="6" t="inlineStr">
-        <is>
-          <t>09/02/2026</t>
-        </is>
-      </c>
-      <c r="F228" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G228" s="6" t="inlineStr">
+      <c r="D229" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E229" s="7" t="inlineStr">
+        <is>
+          <t>10/02/2026</t>
+        </is>
+      </c>
+      <c r="F229" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G229" s="7" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H229" s="7" t="inlineStr">
+        <is>
+          <t>44/60</t>
+        </is>
+      </c>
+      <c r="I229" s="7" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B230" s="7" t="inlineStr">
+        <is>
+          <t>B2E</t>
+        </is>
+      </c>
+      <c r="C230" s="7" t="inlineStr">
+        <is>
+          <t>CHEST</t>
+        </is>
+      </c>
+      <c r="D230" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E230" s="7" t="inlineStr">
+        <is>
+          <t>11/02/2026</t>
+        </is>
+      </c>
+      <c r="F230" s="7" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G230" s="7" t="inlineStr">
         <is>
           <t>2025/2026</t>
         </is>
       </c>
-      <c r="H228" s="6" t="inlineStr">
-        <is>
-          <t>43/60</t>
-        </is>
-      </c>
-      <c r="I228" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B229" s="6" t="inlineStr">
-        <is>
-          <t>B2E</t>
-        </is>
-      </c>
-      <c r="C229" s="6" t="inlineStr">
-        <is>
-          <t>CHEST</t>
-        </is>
-      </c>
-      <c r="D229" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E229" s="6" t="inlineStr">
-        <is>
-          <t>10/02/2026</t>
-        </is>
-      </c>
-      <c r="F229" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G229" s="6" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="H229" s="6" t="inlineStr">
+      <c r="H230" s="7" t="inlineStr">
         <is>
           <t>44/60</t>
         </is>
       </c>
-      <c r="I229" s="6" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B230" s="6" t="inlineStr">
-        <is>
-          <t>B2E</t>
-        </is>
-      </c>
-      <c r="C230" s="6" t="inlineStr">
-        <is>
-          <t>CHEST</t>
-        </is>
-      </c>
-      <c r="D230" s="6" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E230" s="6" t="inlineStr">
-        <is>
-          <t>11/02/2026</t>
-        </is>
-      </c>
-      <c r="F230" s="6" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G230" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H230" s="6" t="inlineStr">
-        <is>
-          <t>44/60</t>
-        </is>
-      </c>
-      <c r="I230" s="6" t="inlineStr">
+      <c r="I230" s="7" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 01:28:42 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>4.9%</t>
+          <t>3.0%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>68.2%</t>
+          <t>71.9%</t>
         </is>
       </c>
     </row>
@@ -1283,22 +1283,22 @@
         <v>53</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>5.7%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>80.3%</t>
+          <t>77.8%</t>
         </is>
       </c>
     </row>
@@ -1361,17 +1361,17 @@
         <v>53</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
@@ -1439,22 +1439,22 @@
         <v>53</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>39.1%</t>
+          <t>40.6%</t>
         </is>
       </c>
     </row>
@@ -1517,22 +1517,22 @@
         <v>52</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>1.9%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>37.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -1595,22 +1595,22 @@
         <v>54</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>72.8%</t>
+          <t>73.3%</t>
         </is>
       </c>
     </row>
@@ -3013,49 +3013,45 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>B2A</t>
         </is>
       </c>
-      <c r="C51" s="8" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D51" s="8" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>09/02/2026</t>
         </is>
       </c>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G51" s="8" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H51" s="8" t="inlineStr">
-        <is>
-          <t>58/66</t>
-        </is>
-      </c>
-      <c r="I51" s="8" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>0/66</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -5093,49 +5089,45 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B99" s="8" t="inlineStr">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C99" s="8" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D99" s="8" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E99" s="8" t="inlineStr">
+      <c r="E99" s="2" t="inlineStr">
         <is>
           <t>09/02/2026</t>
         </is>
       </c>
-      <c r="F99" s="8" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G99" s="8" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H99" s="8" t="inlineStr">
-        <is>
-          <t>48/62</t>
-        </is>
-      </c>
-      <c r="I99" s="8" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr"/>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6997,49 +6989,45 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="8" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B143" s="8" t="inlineStr">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="C143" s="8" t="inlineStr">
+      <c r="C143" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D143" s="8" t="inlineStr">
+      <c r="D143" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E143" s="8" t="inlineStr">
+      <c r="E143" s="2" t="inlineStr">
         <is>
           <t>09/02/2026</t>
         </is>
       </c>
-      <c r="F143" s="8" t="inlineStr">
+      <c r="F143" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G143" s="8" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H143" s="8" t="inlineStr">
-        <is>
-          <t>24/64</t>
-        </is>
-      </c>
-      <c r="I143" s="8" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G143" s="2" t="inlineStr"/>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>0/64</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7865,49 +7853,45 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="8" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B163" s="8" t="inlineStr">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
         <is>
           <t>B2D</t>
         </is>
       </c>
-      <c r="C163" s="8" t="inlineStr">
+      <c r="C163" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D163" s="8" t="inlineStr">
+      <c r="D163" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E163" s="8" t="inlineStr">
+      <c r="E163" s="2" t="inlineStr">
         <is>
           <t>09/02/2026</t>
         </is>
       </c>
-      <c r="F163" s="8" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G163" s="8" t="inlineStr">
-        <is>
-          <t>2024/2025</t>
-        </is>
-      </c>
-      <c r="H163" s="8" t="inlineStr">
-        <is>
-          <t>23/62</t>
-        </is>
-      </c>
-      <c r="I163" s="8" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr"/>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>0/62</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10664,49 +10648,45 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="8" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B228" s="8" t="inlineStr">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
         <is>
           <t>B2E</t>
         </is>
       </c>
-      <c r="C228" s="8" t="inlineStr">
+      <c r="C228" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D228" s="8" t="inlineStr">
+      <c r="D228" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E228" s="8" t="inlineStr">
+      <c r="E228" s="2" t="inlineStr">
         <is>
           <t>09/02/2026</t>
         </is>
       </c>
-      <c r="F228" s="8" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G228" s="8" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H228" s="8" t="inlineStr">
-        <is>
-          <t>43/60</t>
-        </is>
-      </c>
-      <c r="I228" s="8" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr"/>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>0/60</t>
+        </is>
+      </c>
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>